<commit_message>
WP-R3: regenera golden (docs/evidencia_p0/golden) tras los cambios deliberados
30 diferencias, todas explicadas: config (espera_dce 30->0, espera_tome 30->60, revision_textos 3->4,
PROX_AUDIENCIA «decretada», scope HISTORIA, _meta.version v9.2.0) y 3 filas de Espera con
HISTORIA.E05_DIAS («Al 8 de octubre de 2026, RUS registra N días de espera.»).
Verificación: PARIDAD PASÓ contra el golden regenerado.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017uPaxcgXhUC1UXn6NTTVNa
</commit_message>
<xml_diff>
--- a/docs/evidencia_p0/golden/Observaciones_ESPERA.xlsx
+++ b/docs/evidencia_p0/golden/Observaciones_ESPERA.xlsx
@@ -606,17 +606,17 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>["ESPERA.E05_PROYECTO_Y_CORREO"]</t>
+          <t>["ESPERA.E05_PROYECTO_Y_CORREO", "HISTORIA.E05_DIAS"]</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
+          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
         </is>
       </c>
     </row>
@@ -686,17 +686,17 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>["ESPERA.E05_SOLO_CORREO"]</t>
+          <t>["ESPERA.E05_SOLO_CORREO", "HISTORIA.E05_DIAS"]</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
+          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
         </is>
       </c>
     </row>
@@ -766,17 +766,17 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>["ESPERA.E05_PROYECTO_Y_CORREO"]</t>
+          <t>["ESPERA.E05_PROYECTO_Y_CORREO", "HISTORIA.E05_DIAS"]</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
+          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
         </is>
       </c>
     </row>
@@ -982,12 +982,12 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>["ESPERA.E05_PROYECTO_Y_CORREO"]</t>
+          <t>["ESPERA.E05_PROYECTO_Y_CORREO", "HISTORIA.E05_DIAS"]</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1013,12 +1013,12 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>["ESPERA.E05_SOLO_CORREO"]</t>
+          <t>["ESPERA.E05_SOLO_CORREO", "HISTORIA.E05_DIAS"]</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1044,12 +1044,12 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>["ESPERA.E05_PROYECTO_Y_CORREO"]</t>
+          <t>["ESPERA.E05_PROYECTO_Y_CORREO", "HISTORIA.E05_DIAS"]</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">

</xml_diff>

<commit_message>
Decisión x: orden por grupo, un dato una vez y reglas de prórroga, ingreso, curador y causa (WP-65)
- Orden transversal en Espera, Cumplimiento e Informes: constancias, acciones del Centro, gestión del Tribunal.
- Prórroga con 'hasta', marca prioritaria (90 días) y silencio si la bitácora ya la mencionó.
- Ingreso efectivo con ventana de 30 días; 'Ing.Serv.' como resolución de ingreso (cierra el folio por fecha).
- Curador solo si RUS no lo tiene (nivel 2); aclaración de causa transversal; oído y bitácora.
- Egreso posterior a la mayoría de edad; E10 reemplaza los días de espera; C8 breve; textos 'de que'.
- TEXT_REVISION 5 con migración, historia-3, golden regenerado de forma deliberada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VB84tpYXBaUxLxFtBYLGQx
</commit_message>
<xml_diff>
--- a/docs/evidencia_p0/golden/Observaciones_ESPERA.xlsx
+++ b/docs/evidencia_p0/golden/Observaciones_ESPERA.xlsx
@@ -611,12 +611,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
+          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
         </is>
       </c>
     </row>
@@ -691,12 +691,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
+          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
+          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
+          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona DCE: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite correo al programa consultando fecha estimada de ingreso.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
         </is>
       </c>
     </row>
@@ -771,12 +771,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 60 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 60 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -786,7 +786,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
+          <t>{"decisions": {"mail": {}, "resolution": "auto", "structured": true}, "excluded": false, "overrides": {}, "proposal": "Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 60 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.", "resolution_cell": "", "version": 1, "word_overrides": {}}</t>
         </is>
       </c>
     </row>
@@ -982,7 +982,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1013,7 +1013,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Se remite correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 30 días de espera.</t>
+          <t>Persona DCE: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1044,7 +1044,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso. Al 8 de octubre de 2026, RUS registra 60 días de espera.</t>
+          <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 60 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">

</xml_diff>

<commit_message>
WP-66: ronda del usuario 16-oct (informes por vencer en el paquete, período de recolección, RES sugerido, búsqueda, formato de resolución, rendimiento)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VB84tpYXBaUxLxFtBYLGQx
</commit_message>
<xml_diff>
--- a/docs/evidencia_p0/golden/Observaciones_ESPERA.xlsx
+++ b/docs/evidencia_p0/golden/Observaciones_ESPERA.xlsx
@@ -619,6 +619,11 @@
           <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 30 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
         </is>
       </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>PC_IE</t>
+        </is>
+      </c>
       <c r="U2" t="inlineStr">
         <is>
           <t>PROPUESTA</t>
@@ -777,6 +782,11 @@
       <c r="P4" t="inlineStr">
         <is>
           <t>Persona AFT: Medida revisada, a la espera de ingreso efectivo. Al 8 de octubre de 2026, RUS registra 60 días de espera. Se remite proyecto de resolución pidiendo cuenta del ingreso efectivo y correo al programa consultando fecha estimada de ingreso.</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>PC_IE</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">

</xml_diff>